<commit_message>
Finish Kaeya Remap and Add VG Remap Tutorial
</commit_message>
<xml_diff>
--- a/Data/RemapDrafts/KaeyaRemapDraft.xlsx
+++ b/Data/RemapDrafts/KaeyaRemapDraft.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Computer\Games\Genshin\Repos\Repos\Fix-Raiden-Boss\Data\RemapDrafts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E393708D-60F3-47E9-81F3-836FC9251300}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4C2DA4-DEE6-4BA0-8973-9F46B7AF7E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" activeTab="1" xr2:uid="{2D312B7B-4EF7-45D3-A72D-D9B2BCB5622F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="34620" windowHeight="13900" activeTab="1" xr2:uid="{2D312B7B-4EF7-45D3-A72D-D9B2BCB5622F}"/>
   </bookViews>
   <sheets>
     <sheet name="Credits" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'V4.0 - Kaeya to KaeyaSailwind'!$A$1:$D$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'V4.0 - KaeyaSailwind to Kaeya'!$A$1:$D$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="51">
   <si>
     <t>Authors</t>
   </si>
@@ -140,6 +141,60 @@
   </si>
   <si>
     <t>Kaeya's vision</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's ponytail</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right upper arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwinds's fur</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right middle arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left upper arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left middle arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right shoulder</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right foot</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right lower arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right calf</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's right toes</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left calf</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left shoulder</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left foot</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left lower arm</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left thigh</t>
+  </si>
+  <si>
+    <t>KaeyaSailwind's left toes</t>
+  </si>
+  <si>
+    <t>Kaeya's left thigh</t>
   </si>
 </sst>
 </file>
@@ -210,7 +265,17 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -552,22 +617,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA5E3300-FDE5-46D0-8524-5C9724E399BE}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:1" ht="26" x14ac:dyDescent="0.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -583,15 +648,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE905EB-47CE-442F-82D7-1D68299253F1}">
   <dimension ref="A1:D88"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="105.42578125" customWidth="1"/>
+    <col min="1" max="1" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="105.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>5</v>
       </c>
@@ -605,7 +670,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>0</v>
       </c>
@@ -613,7 +678,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -621,7 +686,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2</v>
       </c>
@@ -629,7 +694,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>3</v>
       </c>
@@ -637,7 +702,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>4</v>
       </c>
@@ -645,7 +710,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>5</v>
       </c>
@@ -653,7 +718,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>6</v>
       </c>
@@ -667,7 +732,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>7</v>
       </c>
@@ -678,7 +743,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>8</v>
       </c>
@@ -689,7 +754,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>9</v>
       </c>
@@ -700,7 +765,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>10</v>
       </c>
@@ -711,7 +776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>11</v>
       </c>
@@ -722,7 +787,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>12</v>
       </c>
@@ -733,7 +798,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>13</v>
       </c>
@@ -741,7 +806,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>14</v>
       </c>
@@ -749,7 +814,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>15</v>
       </c>
@@ -757,7 +822,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>16</v>
       </c>
@@ -765,7 +830,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>17</v>
       </c>
@@ -773,7 +838,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>18</v>
       </c>
@@ -781,7 +846,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>19</v>
       </c>
@@ -789,7 +854,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>20</v>
       </c>
@@ -797,7 +862,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>21</v>
       </c>
@@ -805,7 +870,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>22</v>
       </c>
@@ -813,7 +878,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>23</v>
       </c>
@@ -821,7 +886,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>24</v>
       </c>
@@ -829,7 +894,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>25</v>
       </c>
@@ -837,7 +902,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>26</v>
       </c>
@@ -845,7 +910,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>27</v>
       </c>
@@ -853,7 +918,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>28</v>
       </c>
@@ -861,7 +926,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>29</v>
       </c>
@@ -872,7 +937,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>30</v>
       </c>
@@ -880,7 +945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>31</v>
       </c>
@@ -888,7 +953,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>32</v>
       </c>
@@ -896,7 +961,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>33</v>
       </c>
@@ -907,7 +972,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>34</v>
       </c>
@@ -918,7 +983,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>35</v>
       </c>
@@ -929,7 +994,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>36</v>
       </c>
@@ -940,7 +1005,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>37</v>
       </c>
@@ -948,7 +1013,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>38</v>
       </c>
@@ -956,7 +1021,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>39</v>
       </c>
@@ -964,7 +1029,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>40</v>
       </c>
@@ -972,7 +1037,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>41</v>
       </c>
@@ -980,7 +1045,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>42</v>
       </c>
@@ -988,7 +1053,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>43</v>
       </c>
@@ -996,7 +1061,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>44</v>
       </c>
@@ -1004,7 +1069,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>45</v>
       </c>
@@ -1012,7 +1077,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>46</v>
       </c>
@@ -1020,7 +1085,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>47</v>
       </c>
@@ -1028,7 +1093,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>48</v>
       </c>
@@ -1036,7 +1101,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>49</v>
       </c>
@@ -1044,7 +1109,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>50</v>
       </c>
@@ -1052,7 +1117,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>51</v>
       </c>
@@ -1060,7 +1125,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>52</v>
       </c>
@@ -1068,7 +1133,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>53</v>
       </c>
@@ -1082,7 +1147,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>54</v>
       </c>
@@ -1093,7 +1158,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>55</v>
       </c>
@@ -1107,7 +1172,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>56</v>
       </c>
@@ -1118,7 +1183,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>57</v>
       </c>
@@ -1129,7 +1194,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>58</v>
       </c>
@@ -1143,7 +1208,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>59</v>
       </c>
@@ -1154,7 +1219,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>60</v>
       </c>
@@ -1162,7 +1227,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>61</v>
       </c>
@@ -1176,7 +1241,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>62</v>
       </c>
@@ -1187,7 +1252,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>63</v>
       </c>
@@ -1198,7 +1263,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>64</v>
       </c>
@@ -1212,7 +1277,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>65</v>
       </c>
@@ -1223,7 +1288,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>66</v>
       </c>
@@ -1237,7 +1302,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>67</v>
       </c>
@@ -1248,7 +1313,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>68</v>
       </c>
@@ -1259,7 +1324,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>69</v>
       </c>
@@ -1270,7 +1335,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>70</v>
       </c>
@@ -1281,7 +1346,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>71</v>
       </c>
@@ -1292,7 +1357,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>72</v>
       </c>
@@ -1303,7 +1368,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>73</v>
       </c>
@@ -1311,7 +1376,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>74</v>
       </c>
@@ -1319,7 +1384,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>75</v>
       </c>
@@ -1327,7 +1392,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>76</v>
       </c>
@@ -1335,7 +1400,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>77</v>
       </c>
@@ -1346,7 +1411,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>78</v>
       </c>
@@ -1357,7 +1422,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>79</v>
       </c>
@@ -1368,7 +1433,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>80</v>
       </c>
@@ -1379,15 +1444,18 @@
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>81</v>
       </c>
       <c r="B83">
         <v>62</v>
       </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D83" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>82</v>
       </c>
@@ -1398,7 +1466,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>83</v>
       </c>
@@ -1409,7 +1477,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>84</v>
       </c>
@@ -1420,7 +1488,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>85</v>
       </c>
@@ -1431,7 +1499,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>86</v>
       </c>
@@ -1442,17 +1510,682 @@
   </sheetData>
   <autoFilter ref="A1:D88" xr:uid="{9EE905EB-47CE-442F-82D7-1D68299253F1}"/>
   <conditionalFormatting sqref="B2:B88">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AB5BB81-FABE-4E71-87CA-B491B54DCB56}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:D74"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="77.54296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>69</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>11</v>
+      </c>
+      <c r="B13">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15">
+        <v>13</v>
+      </c>
+      <c r="B15">
+        <v>64</v>
+      </c>
+      <c r="C15">
+        <v>0.1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17">
+        <v>15</v>
+      </c>
+      <c r="B17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18">
+        <v>16</v>
+      </c>
+      <c r="B18">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19">
+        <v>17</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20">
+        <v>18</v>
+      </c>
+      <c r="B20">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21">
+        <v>19</v>
+      </c>
+      <c r="B21">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="B22">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23">
+        <v>21</v>
+      </c>
+      <c r="B23">
+        <v>10</v>
+      </c>
+      <c r="D23" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24">
+        <v>22</v>
+      </c>
+      <c r="B24">
+        <v>35</v>
+      </c>
+      <c r="D24" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25">
+        <v>23</v>
+      </c>
+      <c r="B25">
+        <v>34</v>
+      </c>
+      <c r="D25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26">
+        <v>24</v>
+      </c>
+      <c r="B26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27">
+        <v>25</v>
+      </c>
+      <c r="B27">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28">
+        <v>26</v>
+      </c>
+      <c r="B28">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29">
+        <v>27</v>
+      </c>
+      <c r="B29">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30">
+        <v>28</v>
+      </c>
+      <c r="B30">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31">
+        <v>29</v>
+      </c>
+      <c r="B31">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A32">
+        <v>30</v>
+      </c>
+      <c r="B32">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A33">
+        <v>31</v>
+      </c>
+      <c r="B33">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A34">
+        <v>32</v>
+      </c>
+      <c r="B34">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35">
+        <v>33</v>
+      </c>
+      <c r="B35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36">
+        <v>34</v>
+      </c>
+      <c r="B36">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37">
+        <v>35</v>
+      </c>
+      <c r="B37">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38">
+        <v>36</v>
+      </c>
+      <c r="B38">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A39">
+        <v>37</v>
+      </c>
+      <c r="B39">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A40">
+        <v>38</v>
+      </c>
+      <c r="B40">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A41">
+        <v>39</v>
+      </c>
+      <c r="B41">
+        <v>79</v>
+      </c>
+      <c r="D41" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A42">
+        <v>40</v>
+      </c>
+      <c r="B42">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>41</v>
+      </c>
+      <c r="B43">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>42</v>
+      </c>
+      <c r="B44">
+        <v>77</v>
+      </c>
+      <c r="D44" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>43</v>
+      </c>
+      <c r="B45">
+        <v>80</v>
+      </c>
+      <c r="D45" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>44</v>
+      </c>
+      <c r="B46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>45</v>
+      </c>
+      <c r="B47">
+        <v>82</v>
+      </c>
+      <c r="D47" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>46</v>
+      </c>
+      <c r="B48">
+        <v>33</v>
+      </c>
+      <c r="D48" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>47</v>
+      </c>
+      <c r="B49">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>48</v>
+      </c>
+      <c r="B50">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>49</v>
+      </c>
+      <c r="B51">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>50</v>
+      </c>
+      <c r="B52">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>51</v>
+      </c>
+      <c r="B53">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>52</v>
+      </c>
+      <c r="B54">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>53</v>
+      </c>
+      <c r="B55">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>54</v>
+      </c>
+      <c r="B56">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A57">
+        <v>55</v>
+      </c>
+      <c r="B57">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A58">
+        <v>56</v>
+      </c>
+      <c r="B58">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A59">
+        <v>57</v>
+      </c>
+      <c r="B59">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60">
+        <v>58</v>
+      </c>
+      <c r="B60">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61">
+        <v>59</v>
+      </c>
+      <c r="B61">
+        <v>83</v>
+      </c>
+      <c r="D61" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62">
+        <v>60</v>
+      </c>
+      <c r="B62">
+        <v>36</v>
+      </c>
+      <c r="D62" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63">
+        <v>61</v>
+      </c>
+      <c r="B63">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64">
+        <v>62</v>
+      </c>
+      <c r="B64">
+        <v>81</v>
+      </c>
+      <c r="D64" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65">
+        <v>63</v>
+      </c>
+      <c r="B65">
+        <v>84</v>
+      </c>
+      <c r="D65" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66">
+        <v>64</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67">
+        <v>65</v>
+      </c>
+      <c r="B67">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68">
+        <v>66</v>
+      </c>
+      <c r="B68">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69">
+        <v>67</v>
+      </c>
+      <c r="B69">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70">
+        <v>68</v>
+      </c>
+      <c r="B70">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71">
+        <v>69</v>
+      </c>
+      <c r="B71">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72">
+        <v>70</v>
+      </c>
+      <c r="B72">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73">
+        <v>71</v>
+      </c>
+      <c r="B73">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74">
+        <v>72</v>
+      </c>
+      <c r="B74">
+        <v>52</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D1" xr:uid="{8AB5BB81-FABE-4E71-87CA-B491B54DCB56}"/>
+  <conditionalFormatting sqref="B2:B88">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>